<commit_message>
Add data traps (cp1252 extract, NBSP, accented term) + per-file encoding detection; new seeded spec defects
</commit_message>
<xml_diff>
--- a/examples/sdtm/spec_draft.xlsx
+++ b/examples/sdtm/spec_draft.xlsx
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Map RAW_DM.RAND_ARM using codelist ARM; if missing set to 'Screen Failure'</t>
+          <t>Map RAW_DM.RAND_ARM using codelist ARM; if missing set to 'Screen Failure"</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Set to 'AE'</t>
+          <t>Set to ‘AE’</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>

</xml_diff>